<commit_message>
Fix: PPR can never display below Half-PPR for the same player
</commit_message>
<xml_diff>
--- a/workbook.xlsx
+++ b/workbook.xlsx
@@ -2664,7 +2664,7 @@
       </c>
       <c r="E53" s="6" t="n">
         <f aca="false">RB!V17</f>
-        <v>42.9</v>
+        <v>42.3</v>
       </c>
       <c r="F53" s="7" t="n">
         <f aca="false">RB!W17</f>
@@ -2889,7 +2889,7 @@
       </c>
       <c r="E62" s="6" t="n">
         <f aca="false">RB!V26</f>
-        <v>23.8</v>
+        <v>23.1</v>
       </c>
       <c r="F62" s="7" t="n">
         <f aca="false">RB!W26</f>
@@ -2964,7 +2964,7 @@
       </c>
       <c r="E65" s="6" t="n">
         <f aca="false">RB!V29</f>
-        <v>20.9</v>
+        <v>20.3</v>
       </c>
       <c r="F65" s="7" t="n">
         <f aca="false">RB!W29</f>
@@ -3064,7 +3064,7 @@
       </c>
       <c r="E69" s="6" t="n">
         <f aca="false">RB!V33</f>
-        <v>15</v>
+        <v>14.9</v>
       </c>
       <c r="F69" s="7" t="n">
         <f aca="false">RB!W33</f>
@@ -3214,7 +3214,7 @@
       </c>
       <c r="E75" s="6" t="n">
         <f aca="false">RB!V39</f>
-        <v>10.6</v>
+        <v>9.5</v>
       </c>
       <c r="F75" s="7" t="n">
         <f aca="false">RB!W39</f>
@@ -3289,7 +3289,7 @@
       </c>
       <c r="E78" s="6" t="n">
         <f aca="false">RB!V42</f>
-        <v>10.5</v>
+        <v>8.9</v>
       </c>
       <c r="F78" s="7" t="n">
         <f aca="false">RB!W42</f>
@@ -3364,7 +3364,7 @@
       </c>
       <c r="E81" s="6" t="n">
         <f aca="false">RB!V45</f>
-        <v>8.2</v>
+        <v>8</v>
       </c>
       <c r="F81" s="7" t="n">
         <f aca="false">RB!W45</f>
@@ -3414,7 +3414,7 @@
       </c>
       <c r="E83" s="6" t="n">
         <f aca="false">RB!V47</f>
-        <v>6.6</v>
+        <v>5.9</v>
       </c>
       <c r="F83" s="7" t="n">
         <f aca="false">RB!W47</f>
@@ -3464,7 +3464,7 @@
       </c>
       <c r="E85" s="6" t="n">
         <f aca="false">RB!V49</f>
-        <v>4.7</v>
+        <v>4.6</v>
       </c>
       <c r="F85" s="7" t="n">
         <f aca="false">RB!W49</f>
@@ -3514,7 +3514,7 @@
       </c>
       <c r="E87" s="6" t="n">
         <f aca="false">RB!V51</f>
-        <v>4</v>
+        <v>3.9</v>
       </c>
       <c r="F87" s="7" t="n">
         <f aca="false">RB!W51</f>
@@ -3589,7 +3589,7 @@
       </c>
       <c r="E90" s="6" t="n">
         <f aca="false">RB!V54</f>
-        <v>3.8</v>
+        <v>3.6</v>
       </c>
       <c r="F90" s="7" t="n">
         <f aca="false">RB!W54</f>
@@ -3614,7 +3614,7 @@
       </c>
       <c r="E91" s="6" t="n">
         <f aca="false">RB!V55</f>
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
       <c r="F91" s="7" t="n">
         <f aca="false">RB!W55</f>
@@ -3639,7 +3639,7 @@
       </c>
       <c r="E92" s="6" t="n">
         <f aca="false">RB!V56</f>
-        <v>4.2</v>
+        <v>3.5</v>
       </c>
       <c r="F92" s="7" t="n">
         <f aca="false">RB!W56</f>
@@ -3664,7 +3664,7 @@
       </c>
       <c r="E93" s="6" t="n">
         <f aca="false">RB!V57</f>
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="F93" s="7" t="n">
         <f aca="false">RB!W57</f>
@@ -3689,7 +3689,7 @@
       </c>
       <c r="E94" s="6" t="n">
         <f aca="false">RB!V58</f>
-        <v>3.7</v>
+        <v>3.1</v>
       </c>
       <c r="F94" s="7" t="n">
         <f aca="false">RB!W58</f>
@@ -3714,7 +3714,7 @@
       </c>
       <c r="E95" s="6" t="n">
         <f aca="false">RB!V59</f>
-        <v>3.6</v>
+        <v>3</v>
       </c>
       <c r="F95" s="7" t="n">
         <f aca="false">RB!W59</f>
@@ -3764,7 +3764,7 @@
       </c>
       <c r="E97" s="6" t="n">
         <f aca="false">RB!V61</f>
-        <v>2.9</v>
+        <v>2.8</v>
       </c>
       <c r="F97" s="7" t="n">
         <f aca="false">RB!W61</f>
@@ -3814,7 +3814,7 @@
       </c>
       <c r="E99" s="6" t="n">
         <f aca="false">RB!V63</f>
-        <v>2.5</v>
+        <v>2.3</v>
       </c>
       <c r="F99" s="7" t="n">
         <f aca="false">RB!W63</f>
@@ -3839,7 +3839,7 @@
       </c>
       <c r="E100" s="6" t="n">
         <f aca="false">RB!V64</f>
-        <v>2.4</v>
+        <v>2.2</v>
       </c>
       <c r="F100" s="7" t="n">
         <f aca="false">RB!W64</f>
@@ -3864,7 +3864,7 @@
       </c>
       <c r="E101" s="6" t="n">
         <f aca="false">RB!V65</f>
-        <v>2.3</v>
+        <v>2.1</v>
       </c>
       <c r="F101" s="7" t="n">
         <f aca="false">RB!W65</f>
@@ -3889,7 +3889,7 @@
       </c>
       <c r="E102" s="6" t="n">
         <f aca="false">RB!V66</f>
-        <v>2.9</v>
+        <v>2.1</v>
       </c>
       <c r="F102" s="7" t="n">
         <f aca="false">RB!W66</f>
@@ -3914,7 +3914,7 @@
       </c>
       <c r="E103" s="6" t="n">
         <f aca="false">RB!V67</f>
-        <v>2.2</v>
+        <v>2</v>
       </c>
       <c r="F103" s="7" t="n">
         <f aca="false">RB!W67</f>
@@ -3939,7 +3939,7 @@
       </c>
       <c r="E104" s="6" t="n">
         <f aca="false">RB!V68</f>
-        <v>2.5</v>
+        <v>1.7</v>
       </c>
       <c r="F104" s="7" t="n">
         <f aca="false">RB!W68</f>
@@ -3964,7 +3964,7 @@
       </c>
       <c r="E105" s="6" t="n">
         <f aca="false">RB!V69</f>
-        <v>1.7</v>
+        <v>1.2</v>
       </c>
       <c r="F105" s="7" t="n">
         <f aca="false">RB!W69</f>
@@ -3989,7 +3989,7 @@
       </c>
       <c r="E106" s="6" t="n">
         <f aca="false">RB!V70</f>
-        <v>1.5</v>
+        <v>0.7</v>
       </c>
       <c r="F106" s="7" t="n">
         <f aca="false">RB!W70</f>
@@ -4014,7 +4014,7 @@
       </c>
       <c r="E107" s="6" t="n">
         <f aca="false">RB!V71</f>
-        <v>0.9</v>
+        <v>0.4</v>
       </c>
       <c r="F107" s="7" t="n">
         <f aca="false">RB!W71</f>
@@ -4039,7 +4039,7 @@
       </c>
       <c r="E108" s="6" t="n">
         <f aca="false">RB!V72</f>
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
       <c r="F108" s="7" t="n">
         <f aca="false">RB!W72</f>
@@ -5214,7 +5214,7 @@
       </c>
       <c r="E158" s="6" t="n">
         <f aca="false">WR!V46</f>
-        <v>12.3</v>
+        <v>11.6</v>
       </c>
       <c r="F158" s="7" t="n">
         <f aca="false">WR!W46</f>
@@ -5239,7 +5239,7 @@
       </c>
       <c r="E159" s="6" t="n">
         <f aca="false">WR!V47</f>
-        <v>12.5</v>
+        <v>11.5</v>
       </c>
       <c r="F159" s="7" t="n">
         <f aca="false">WR!W47</f>
@@ -5289,7 +5289,7 @@
       </c>
       <c r="E161" s="6" t="n">
         <f aca="false">WR!V49</f>
-        <v>11.5</v>
+        <v>10.8</v>
       </c>
       <c r="F161" s="7" t="n">
         <f aca="false">WR!W49</f>
@@ -5414,7 +5414,7 @@
       </c>
       <c r="E166" s="6" t="n">
         <f aca="false">WR!V54</f>
-        <v>8.9</v>
+        <v>8.2</v>
       </c>
       <c r="F166" s="7" t="n">
         <f aca="false">WR!W54</f>
@@ -5514,7 +5514,7 @@
       </c>
       <c r="E170" s="6" t="n">
         <f aca="false">WR!V58</f>
-        <v>7.4</v>
+        <v>6.9</v>
       </c>
       <c r="F170" s="7" t="n">
         <f aca="false">WR!W58</f>
@@ -5539,7 +5539,7 @@
       </c>
       <c r="E171" s="6" t="n">
         <f aca="false">WR!V59</f>
-        <v>7.3</v>
+        <v>6.6</v>
       </c>
       <c r="F171" s="7" t="n">
         <f aca="false">WR!W59</f>
@@ -5564,7 +5564,7 @@
       </c>
       <c r="E172" s="6" t="n">
         <f aca="false">WR!V60</f>
-        <v>7</v>
+        <v>6.2</v>
       </c>
       <c r="F172" s="7" t="n">
         <f aca="false">WR!W60</f>
@@ -5589,7 +5589,7 @@
       </c>
       <c r="E173" s="6" t="n">
         <f aca="false">WR!V61</f>
-        <v>6.8</v>
+        <v>5.9</v>
       </c>
       <c r="F173" s="7" t="n">
         <f aca="false">WR!W61</f>
@@ -5614,7 +5614,7 @@
       </c>
       <c r="E174" s="6" t="n">
         <f aca="false">WR!V62</f>
-        <v>6.4</v>
+        <v>5.7</v>
       </c>
       <c r="F174" s="7" t="n">
         <f aca="false">WR!W62</f>
@@ -5689,7 +5689,7 @@
       </c>
       <c r="E177" s="6" t="n">
         <f aca="false">WR!V65</f>
-        <v>5.6</v>
+        <v>4.9</v>
       </c>
       <c r="F177" s="7" t="n">
         <f aca="false">WR!W65</f>
@@ -5739,7 +5739,7 @@
       </c>
       <c r="E179" s="6" t="n">
         <f aca="false">WR!V67</f>
-        <v>4.3</v>
+        <v>3.9</v>
       </c>
       <c r="F179" s="7" t="n">
         <f aca="false">WR!W67</f>
@@ -5764,7 +5764,7 @@
       </c>
       <c r="E180" s="6" t="n">
         <f aca="false">WR!V68</f>
-        <v>4.3</v>
+        <v>3.9</v>
       </c>
       <c r="F180" s="7" t="n">
         <f aca="false">WR!W68</f>
@@ -5839,7 +5839,7 @@
       </c>
       <c r="E183" s="6" t="n">
         <f aca="false">WR!V71</f>
-        <v>3.9</v>
+        <v>3.2</v>
       </c>
       <c r="F183" s="7" t="n">
         <f aca="false">WR!W71</f>
@@ -5864,7 +5864,7 @@
       </c>
       <c r="E184" s="6" t="n">
         <f aca="false">WR!V72</f>
-        <v>3.7</v>
+        <v>3</v>
       </c>
       <c r="F184" s="7" t="n">
         <f aca="false">WR!W72</f>
@@ -5914,7 +5914,7 @@
       </c>
       <c r="E186" s="6" t="n">
         <f aca="false">WR!V74</f>
-        <v>3.5</v>
+        <v>2.8</v>
       </c>
       <c r="F186" s="7" t="n">
         <f aca="false">WR!W74</f>
@@ -5939,7 +5939,7 @@
       </c>
       <c r="E187" s="6" t="n">
         <f aca="false">WR!V75</f>
-        <v>3</v>
+        <v>2.4</v>
       </c>
       <c r="F187" s="7" t="n">
         <f aca="false">WR!W75</f>
@@ -5989,7 +5989,7 @@
       </c>
       <c r="E189" s="6" t="n">
         <f aca="false">WR!V77</f>
-        <v>2.2</v>
+        <v>1.6</v>
       </c>
       <c r="F189" s="7" t="n">
         <f aca="false">WR!W77</f>
@@ -6014,7 +6014,7 @@
       </c>
       <c r="E190" s="6" t="n">
         <f aca="false">WR!V78</f>
-        <v>1.8</v>
+        <v>1.4</v>
       </c>
       <c r="F190" s="7" t="n">
         <f aca="false">WR!W78</f>
@@ -6039,7 +6039,7 @@
       </c>
       <c r="E191" s="6" t="n">
         <f aca="false">WR!V79</f>
-        <v>1.9</v>
+        <v>1.2</v>
       </c>
       <c r="F191" s="7" t="n">
         <f aca="false">WR!W79</f>
@@ -6064,7 +6064,7 @@
       </c>
       <c r="E192" s="6" t="n">
         <f aca="false">WR!V80</f>
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="F192" s="7" t="n">
         <f aca="false">WR!W80</f>
@@ -6089,7 +6089,7 @@
       </c>
       <c r="E193" s="6" t="n">
         <f aca="false">WR!V81</f>
-        <v>1.8</v>
+        <v>1.1</v>
       </c>
       <c r="F193" s="7" t="n">
         <f aca="false">WR!W81</f>
@@ -6114,7 +6114,7 @@
       </c>
       <c r="E194" s="6" t="n">
         <f aca="false">WR!V82</f>
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="F194" s="7" t="n">
         <f aca="false">WR!W82</f>
@@ -6139,7 +6139,7 @@
       </c>
       <c r="E195" s="6" t="n">
         <f aca="false">WR!V83</f>
-        <v>1.5</v>
+        <v>0.8</v>
       </c>
       <c r="F195" s="7" t="n">
         <f aca="false">WR!W83</f>
@@ -6164,7 +6164,7 @@
       </c>
       <c r="E196" s="6" t="n">
         <f aca="false">WR!V84</f>
-        <v>1.1</v>
+        <v>0.5</v>
       </c>
       <c r="F196" s="7" t="n">
         <f aca="false">WR!W84</f>
@@ -6189,7 +6189,7 @@
       </c>
       <c r="E197" s="6" t="n">
         <f aca="false">WR!V85</f>
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="F197" s="7" t="n">
         <f aca="false">WR!W85</f>
@@ -6214,7 +6214,7 @@
       </c>
       <c r="E198" s="6" t="n">
         <f aca="false">WR!V86</f>
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="F198" s="7" t="n">
         <f aca="false">WR!W86</f>
@@ -10786,7 +10786,7 @@
         <v>78</v>
       </c>
       <c r="V6" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y6,AA6,AC6,AE6,AG6)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y6,AA6,AC6,AE6,AG6)),1),72.1),"")</f>
         <v>69.9</v>
       </c>
       <c r="W6" s="7" t="n">
@@ -10895,7 +10895,7 @@
         <v>79</v>
       </c>
       <c r="V7" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y7,AA7,AC7,AE7,AG7)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y7,AA7,AC7,AE7,AG7)),1),67.3),"")</f>
         <v>65.4</v>
       </c>
       <c r="W7" s="7" t="n">
@@ -11011,7 +11011,7 @@
         <v>80</v>
       </c>
       <c r="V8" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y8,AA8,AC8,AE8,AG8)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y8,AA8,AC8,AE8,AG8)),1),59.3),"")</f>
         <v>58.2</v>
       </c>
       <c r="W8" s="7" t="n">
@@ -11127,7 +11127,7 @@
         <v>81</v>
       </c>
       <c r="V9" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y9,AA9,AC9,AE9,AG9)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y9,AA9,AC9,AE9,AG9)),1),58.1),"")</f>
         <v>57.4</v>
       </c>
       <c r="W9" s="7" t="n">
@@ -11243,7 +11243,7 @@
         <v>82</v>
       </c>
       <c r="V10" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y10,AA10,AC10,AE10,AG10)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y10,AA10,AC10,AE10,AG10)),1),56.6),"")</f>
         <v>54.4</v>
       </c>
       <c r="W10" s="7" t="n">
@@ -11359,7 +11359,7 @@
         <v>83</v>
       </c>
       <c r="V11" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y11,AA11,AC11,AE11,AG11)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y11,AA11,AC11,AE11,AG11)),1),53.2),"")</f>
         <v>51.4</v>
       </c>
       <c r="W11" s="7" t="n">
@@ -11475,7 +11475,7 @@
         <v>84</v>
       </c>
       <c r="V12" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y12,AA12,AC12,AE12,AG12)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y12,AA12,AC12,AE12,AG12)),1),50.3),"")</f>
         <v>49.7</v>
       </c>
       <c r="W12" s="7" t="n">
@@ -11591,7 +11591,7 @@
         <v>85</v>
       </c>
       <c r="V13" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y13,AA13,AC13,AE13,AG13)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y13,AA13,AC13,AE13,AG13)),1),49.1),"")</f>
         <v>48.5</v>
       </c>
       <c r="W13" s="7" t="n">
@@ -11707,7 +11707,7 @@
         <v>86</v>
       </c>
       <c r="V14" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y14,AA14,AC14,AE14,AG14)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y14,AA14,AC14,AE14,AG14)),1),48.5),"")</f>
         <v>46.5</v>
       </c>
       <c r="W14" s="7" t="n">
@@ -11823,7 +11823,7 @@
         <v>87</v>
       </c>
       <c r="V15" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y15,AA15,AC15,AE15,AG15)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y15,AA15,AC15,AE15,AG15)),1),47.3),"")</f>
         <v>46.2</v>
       </c>
       <c r="W15" s="7" t="n">
@@ -11939,7 +11939,7 @@
         <v>88</v>
       </c>
       <c r="V16" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y16,AA16,AC16,AE16,AG16)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y16,AA16,AC16,AE16,AG16)),1),43.4),"")</f>
         <v>42</v>
       </c>
       <c r="W16" s="7" t="n">
@@ -12055,8 +12055,8 @@
         <v>89</v>
       </c>
       <c r="V17" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y17,AA17,AC17,AE17,AG17)),1),"")</f>
-        <v>42.9</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y17,AA17,AC17,AE17,AG17)),1),42.3),"")</f>
+        <v>42.3</v>
       </c>
       <c r="W17" s="7" t="n">
         <f aca="false">COUNT(X17,Z17,AB17,AD17,AF17)</f>
@@ -12171,7 +12171,7 @@
         <v>90</v>
       </c>
       <c r="V18" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y18,AA18,AC18,AE18,AG18)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y18,AA18,AC18,AE18,AG18)),1),36.6),"")</f>
         <v>35.9</v>
       </c>
       <c r="W18" s="7" t="n">
@@ -12280,7 +12280,7 @@
         <v>91</v>
       </c>
       <c r="V19" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y19,AA19,AC19,AE19,AG19)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y19,AA19,AC19,AE19,AG19)),1),35.3),"")</f>
         <v>34.9</v>
       </c>
       <c r="W19" s="7" t="n">
@@ -12382,7 +12382,7 @@
         <v>92</v>
       </c>
       <c r="V20" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y20,AA20,AC20,AE20,AG20)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y20,AA20,AC20,AE20,AG20)),1),35.2),"")</f>
         <v>34.6</v>
       </c>
       <c r="W20" s="7" t="n">
@@ -12484,7 +12484,7 @@
         <v>93</v>
       </c>
       <c r="V21" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y21,AA21,AC21,AE21,AG21)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y21,AA21,AC21,AE21,AG21)),1),34),"")</f>
         <v>33.2</v>
       </c>
       <c r="W21" s="7" t="n">
@@ -12586,7 +12586,7 @@
         <v>94</v>
       </c>
       <c r="V22" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y22,AA22,AC22,AE22,AG22)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y22,AA22,AC22,AE22,AG22)),1),33),"")</f>
         <v>32.1</v>
       </c>
       <c r="W22" s="7" t="n">
@@ -12688,7 +12688,7 @@
         <v>95</v>
       </c>
       <c r="V23" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y23,AA23,AC23,AE23,AG23)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y23,AA23,AC23,AE23,AG23)),1),30.7),"")</f>
         <v>30.4</v>
       </c>
       <c r="W23" s="7" t="n">
@@ -12790,7 +12790,7 @@
         <v>96</v>
       </c>
       <c r="V24" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y24,AA24,AC24,AE24,AG24)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y24,AA24,AC24,AE24,AG24)),1),25.4),"")</f>
         <v>24.3</v>
       </c>
       <c r="W24" s="7" t="n">
@@ -12892,7 +12892,7 @@
         <v>97</v>
       </c>
       <c r="V25" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y25,AA25,AC25,AE25,AG25)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y25,AA25,AC25,AE25,AG25)),1),24.7),"")</f>
         <v>23.9</v>
       </c>
       <c r="W25" s="7" t="n">
@@ -12994,8 +12994,8 @@
         <v>98</v>
       </c>
       <c r="V26" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y26,AA26,AC26,AE26,AG26)),1),"")</f>
-        <v>23.8</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y26,AA26,AC26,AE26,AG26)),1),23.1),"")</f>
+        <v>23.1</v>
       </c>
       <c r="W26" s="7" t="n">
         <f aca="false">COUNT(X26,Z26,AB26,AD26,AF26)</f>
@@ -13096,7 +13096,7 @@
         <v>99</v>
       </c>
       <c r="V27" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y27,AA27,AC27,AE27,AG27)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y27,AA27,AC27,AE27,AG27)),1),22.5),"")</f>
         <v>22.3</v>
       </c>
       <c r="W27" s="7" t="n">
@@ -13198,7 +13198,7 @@
         <v>100</v>
       </c>
       <c r="V28" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y28,AA28,AC28,AE28,AG28)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y28,AA28,AC28,AE28,AG28)),1),22),"")</f>
         <v>21.9</v>
       </c>
       <c r="W28" s="7" t="n">
@@ -13300,8 +13300,8 @@
         <v>101</v>
       </c>
       <c r="V29" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y29,AA29,AC29,AE29,AG29)),1),"")</f>
-        <v>20.9</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y29,AA29,AC29,AE29,AG29)),1),20.3),"")</f>
+        <v>20.3</v>
       </c>
       <c r="W29" s="7" t="n">
         <f aca="false">COUNT(X29,Z29,AB29,AD29,AF29)</f>
@@ -13402,7 +13402,7 @@
         <v>102</v>
       </c>
       <c r="V30" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y30,AA30,AC30,AE30,AG30)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y30,AA30,AC30,AE30,AG30)),1),18.8),"")</f>
         <v>18</v>
       </c>
       <c r="W30" s="7" t="n">
@@ -13504,7 +13504,7 @@
         <v>103</v>
       </c>
       <c r="V31" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y31,AA31,AC31,AE31,AG31)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y31,AA31,AC31,AE31,AG31)),1),15.8),"")</f>
         <v>14.9</v>
       </c>
       <c r="W31" s="7" t="n">
@@ -13606,7 +13606,7 @@
         <v>104</v>
       </c>
       <c r="V32" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y32,AA32,AC32,AE32,AG32)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y32,AA32,AC32,AE32,AG32)),1),15.5),"")</f>
         <v>14.5</v>
       </c>
       <c r="W32" s="7" t="n">
@@ -13708,8 +13708,8 @@
         <v>105</v>
       </c>
       <c r="V33" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y33,AA33,AC33,AE33,AG33)),1),"")</f>
-        <v>15</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y33,AA33,AC33,AE33,AG33)),1),14.9),"")</f>
+        <v>14.9</v>
       </c>
       <c r="W33" s="7" t="n">
         <f aca="false">COUNT(X33,Z33,AB33,AD33,AF33)</f>
@@ -13810,7 +13810,7 @@
         <v>106</v>
       </c>
       <c r="V34" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y34,AA34,AC34,AE34,AG34)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y34,AA34,AC34,AE34,AG34)),1),14.4),"")</f>
         <v>14.4</v>
       </c>
       <c r="W34" s="7" t="n">
@@ -13912,7 +13912,7 @@
         <v>107</v>
       </c>
       <c r="V35" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y35,AA35,AC35,AE35,AG35)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y35,AA35,AC35,AE35,AG35)),1),13.6),"")</f>
         <v>13.3</v>
       </c>
       <c r="W35" s="7" t="n">
@@ -14012,7 +14012,7 @@
         <v>108</v>
       </c>
       <c r="V36" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y36,AA36,AC36,AE36,AG36)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y36,AA36,AC36,AE36,AG36)),1),11.8),"")</f>
         <v>9.7</v>
       </c>
       <c r="W36" s="7" t="n">
@@ -14112,7 +14112,7 @@
         <v>109</v>
       </c>
       <c r="V37" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y37,AA37,AC37,AE37,AG37)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y37,AA37,AC37,AE37,AG37)),1),11),"")</f>
         <v>11</v>
       </c>
       <c r="W37" s="7" t="n">
@@ -14212,7 +14212,7 @@
         <v>110</v>
       </c>
       <c r="V38" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y38,AA38,AC38,AE38,AG38)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y38,AA38,AC38,AE38,AG38)),1),10.3),"")</f>
         <v>9.7</v>
       </c>
       <c r="W38" s="7" t="n">
@@ -14310,8 +14310,8 @@
         <v>111</v>
       </c>
       <c r="V39" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y39,AA39,AC39,AE39,AG39)),1),"")</f>
-        <v>10.6</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y39,AA39,AC39,AE39,AG39)),1),9.5),"")</f>
+        <v>9.5</v>
       </c>
       <c r="W39" s="7" t="n">
         <f aca="false">COUNT(X39,Z39,AB39,AD39,AF39)</f>
@@ -14410,7 +14410,7 @@
         <v>112</v>
       </c>
       <c r="V40" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y40,AA40,AC40,AE40,AG40)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y40,AA40,AC40,AE40,AG40)),1),9.3),"")</f>
         <v>8.5</v>
       </c>
       <c r="W40" s="7" t="n">
@@ -14512,7 +14512,7 @@
         <v>113</v>
       </c>
       <c r="V41" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y41,AA41,AC41,AE41,AG41)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y41,AA41,AC41,AE41,AG41)),1),9.1),"")</f>
         <v>8.1</v>
       </c>
       <c r="W41" s="7" t="n">
@@ -14612,8 +14612,8 @@
         <v>114</v>
       </c>
       <c r="V42" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y42,AA42,AC42,AE42,AG42)),1),"")</f>
-        <v>10.5</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y42,AA42,AC42,AE42,AG42)),1),8.9),"")</f>
+        <v>8.9</v>
       </c>
       <c r="W42" s="7" t="n">
         <f aca="false">COUNT(X42,Z42,AB42,AD42,AF42)</f>
@@ -14708,7 +14708,7 @@
         <v>115</v>
       </c>
       <c r="V43" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y43,AA43,AC43,AE43,AG43)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y43,AA43,AC43,AE43,AG43)),1),8.4),"")</f>
         <v>6.4</v>
       </c>
       <c r="W43" s="7" t="n">
@@ -14806,7 +14806,7 @@
         <v>116</v>
       </c>
       <c r="V44" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y44,AA44,AC44,AE44,AG44)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y44,AA44,AC44,AE44,AG44)),1),8.2),"")</f>
         <v>7.1</v>
       </c>
       <c r="W44" s="7" t="n">
@@ -14908,8 +14908,8 @@
         <v>117</v>
       </c>
       <c r="V45" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y45,AA45,AC45,AE45,AG45)),1),"")</f>
-        <v>8.2</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y45,AA45,AC45,AE45,AG45)),1),8),"")</f>
+        <v>8</v>
       </c>
       <c r="W45" s="7" t="n">
         <f aca="false">COUNT(X45,Z45,AB45,AD45,AF45)</f>
@@ -15008,7 +15008,7 @@
         <v>118</v>
       </c>
       <c r="V46" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y46,AA46,AC46,AE46,AG46)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y46,AA46,AC46,AE46,AG46)),1),6.3),"")</f>
         <v>1.9</v>
       </c>
       <c r="W46" s="7" t="n">
@@ -15108,8 +15108,8 @@
         <v>119</v>
       </c>
       <c r="V47" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y47,AA47,AC47,AE47,AG47)),1),"")</f>
-        <v>6.6</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y47,AA47,AC47,AE47,AG47)),1),5.9),"")</f>
+        <v>5.9</v>
       </c>
       <c r="W47" s="7" t="n">
         <f aca="false">COUNT(X47,Z47,AB47,AD47,AF47)</f>
@@ -15210,7 +15210,7 @@
         <v>120</v>
       </c>
       <c r="V48" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y48,AA48,AC48,AE48,AG48)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y48,AA48,AC48,AE48,AG48)),1),5.5),"")</f>
         <v>5.2</v>
       </c>
       <c r="W48" s="7" t="n">
@@ -15308,8 +15308,8 @@
         <v>121</v>
       </c>
       <c r="V49" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y49,AA49,AC49,AE49,AG49)),1),"")</f>
-        <v>4.7</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y49,AA49,AC49,AE49,AG49)),1),4.6),"")</f>
+        <v>4.6</v>
       </c>
       <c r="W49" s="7" t="n">
         <f aca="false">COUNT(X49,Z49,AB49,AD49,AF49)</f>
@@ -15404,7 +15404,7 @@
         <v>122</v>
       </c>
       <c r="V50" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y50,AA50,AC50,AE50,AG50)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y50,AA50,AC50,AE50,AG50)),1),4.3),"")</f>
         <v>3.3</v>
       </c>
       <c r="W50" s="7" t="n">
@@ -15500,8 +15500,8 @@
         <v>123</v>
       </c>
       <c r="V51" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y51,AA51,AC51,AE51,AG51)),1),"")</f>
-        <v>4</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y51,AA51,AC51,AE51,AG51)),1),3.9),"")</f>
+        <v>3.9</v>
       </c>
       <c r="W51" s="7" t="n">
         <f aca="false">COUNT(X51,Z51,AB51,AD51,AF51)</f>
@@ -15596,7 +15596,7 @@
         <v>124</v>
       </c>
       <c r="V52" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y52,AA52,AC52,AE52,AG52)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y52,AA52,AC52,AE52,AG52)),1),3.8),"")</f>
         <v>3.4</v>
       </c>
       <c r="W52" s="7" t="n">
@@ -15692,7 +15692,7 @@
         <v>126</v>
       </c>
       <c r="V53" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y53,AA53,AC53,AE53,AG53)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y53,AA53,AC53,AE53,AG53)),1),3.7),"")</f>
         <v>3.2</v>
       </c>
       <c r="W53" s="7" t="n">
@@ -15786,8 +15786,8 @@
         <v>127</v>
       </c>
       <c r="V54" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y54,AA54,AC54,AE54,AG54)),1),"")</f>
-        <v>3.8</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y54,AA54,AC54,AE54,AG54)),1),3.6),"")</f>
+        <v>3.6</v>
       </c>
       <c r="W54" s="7" t="n">
         <f aca="false">COUNT(X54,Z54,AB54,AD54,AF54)</f>
@@ -15880,8 +15880,8 @@
         <v>128</v>
       </c>
       <c r="V55" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y55,AA55,AC55,AE55,AG55)),1),"")</f>
-        <v>3.7</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y55,AA55,AC55,AE55,AG55)),1),3.6),"")</f>
+        <v>3.6</v>
       </c>
       <c r="W55" s="7" t="n">
         <f aca="false">COUNT(X55,Z55,AB55,AD55,AF55)</f>
@@ -15974,8 +15974,8 @@
         <v>129</v>
       </c>
       <c r="V56" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y56,AA56,AC56,AE56,AG56)),1),"")</f>
-        <v>4.2</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y56,AA56,AC56,AE56,AG56)),1),3.5),"")</f>
+        <v>3.5</v>
       </c>
       <c r="W56" s="7" t="n">
         <f aca="false">COUNT(X56,Z56,AB56,AD56,AF56)</f>
@@ -16076,8 +16076,8 @@
         <v>130</v>
       </c>
       <c r="V57" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y57,AA57,AC57,AE57,AG57)),1),"")</f>
-        <v>3.4</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y57,AA57,AC57,AE57,AG57)),1),3.3),"")</f>
+        <v>3.3</v>
       </c>
       <c r="W57" s="7" t="n">
         <f aca="false">COUNT(X57,Z57,AB57,AD57,AF57)</f>
@@ -16170,8 +16170,8 @@
         <v>131</v>
       </c>
       <c r="V58" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y58,AA58,AC58,AE58,AG58)),1),"")</f>
-        <v>3.7</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y58,AA58,AC58,AE58,AG58)),1),3.1),"")</f>
+        <v>3.1</v>
       </c>
       <c r="W58" s="7" t="n">
         <f aca="false">COUNT(X58,Z58,AB58,AD58,AF58)</f>
@@ -16268,8 +16268,8 @@
         <v>132</v>
       </c>
       <c r="V59" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y59,AA59,AC59,AE59,AG59)),1),"")</f>
-        <v>3.6</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y59,AA59,AC59,AE59,AG59)),1),3),"")</f>
+        <v>3</v>
       </c>
       <c r="W59" s="7" t="n">
         <f aca="false">COUNT(X59,Z59,AB59,AD59,AF59)</f>
@@ -16366,7 +16366,7 @@
         <v>133</v>
       </c>
       <c r="V60" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y60,AA60,AC60,AE60,AG60)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y60,AA60,AC60,AE60,AG60)),1),2.9),"")</f>
         <v>2.4</v>
       </c>
       <c r="W60" s="7" t="n">
@@ -16464,8 +16464,8 @@
         <v>134</v>
       </c>
       <c r="V61" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y61,AA61,AC61,AE61,AG61)),1),"")</f>
-        <v>2.9</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y61,AA61,AC61,AE61,AG61)),1),2.8),"")</f>
+        <v>2.8</v>
       </c>
       <c r="W61" s="7" t="n">
         <f aca="false">COUNT(X61,Z61,AB61,AD61,AF61)</f>
@@ -16558,7 +16558,7 @@
         <v>135</v>
       </c>
       <c r="V62" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y62,AA62,AC62,AE62,AG62)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y62,AA62,AC62,AE62,AG62)),1),2.4),"")</f>
         <v>1.9</v>
       </c>
       <c r="W62" s="7" t="n">
@@ -16652,8 +16652,8 @@
         <v>136</v>
       </c>
       <c r="V63" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y63,AA63,AC63,AE63,AG63)),1),"")</f>
-        <v>2.5</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y63,AA63,AC63,AE63,AG63)),1),2.3),"")</f>
+        <v>2.3</v>
       </c>
       <c r="W63" s="7" t="n">
         <f aca="false">COUNT(X63,Z63,AB63,AD63,AF63)</f>
@@ -16746,8 +16746,8 @@
         <v>137</v>
       </c>
       <c r="V64" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y64,AA64,AC64,AE64,AG64)),1),"")</f>
-        <v>2.4</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y64,AA64,AC64,AE64,AG64)),1),2.2),"")</f>
+        <v>2.2</v>
       </c>
       <c r="W64" s="7" t="n">
         <f aca="false">COUNT(X64,Z64,AB64,AD64,AF64)</f>
@@ -16840,8 +16840,8 @@
         <v>138</v>
       </c>
       <c r="V65" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y65,AA65,AC65,AE65,AG65)),1),"")</f>
-        <v>2.3</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y65,AA65,AC65,AE65,AG65)),1),2.1),"")</f>
+        <v>2.1</v>
       </c>
       <c r="W65" s="7" t="n">
         <f aca="false">COUNT(X65,Z65,AB65,AD65,AF65)</f>
@@ -16934,8 +16934,8 @@
         <v>139</v>
       </c>
       <c r="V66" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y66,AA66,AC66,AE66,AG66)),1),"")</f>
-        <v>2.9</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y66,AA66,AC66,AE66,AG66)),1),2.1),"")</f>
+        <v>2.1</v>
       </c>
       <c r="W66" s="7" t="n">
         <f aca="false">COUNT(X66,Z66,AB66,AD66,AF66)</f>
@@ -17030,8 +17030,8 @@
         <v>141</v>
       </c>
       <c r="V67" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y67,AA67,AC67,AE67,AG67)),1),"")</f>
-        <v>2.2</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y67,AA67,AC67,AE67,AG67)),1),2),"")</f>
+        <v>2</v>
       </c>
       <c r="W67" s="7" t="n">
         <f aca="false">COUNT(X67,Z67,AB67,AD67,AF67)</f>
@@ -17126,8 +17126,8 @@
         <v>142</v>
       </c>
       <c r="V68" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y68,AA68,AC68,AE68,AG68)),1),"")</f>
-        <v>2.5</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y68,AA68,AC68,AE68,AG68)),1),1.7),"")</f>
+        <v>1.7</v>
       </c>
       <c r="W68" s="7" t="n">
         <f aca="false">COUNT(X68,Z68,AB68,AD68,AF68)</f>
@@ -17222,8 +17222,8 @@
         <v>143</v>
       </c>
       <c r="V69" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y69,AA69,AC69,AE69,AG69)),1),"")</f>
-        <v>1.7</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y69,AA69,AC69,AE69,AG69)),1),1.2),"")</f>
+        <v>1.2</v>
       </c>
       <c r="W69" s="7" t="n">
         <f aca="false">COUNT(X69,Z69,AB69,AD69,AF69)</f>
@@ -17318,8 +17318,8 @@
         <v>144</v>
       </c>
       <c r="V70" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y70,AA70,AC70,AE70,AG70)),1),"")</f>
-        <v>1.5</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y70,AA70,AC70,AE70,AG70)),1),0.7),"")</f>
+        <v>0.7</v>
       </c>
       <c r="W70" s="7" t="n">
         <f aca="false">COUNT(X70,Z70,AB70,AD70,AF70)</f>
@@ -17414,8 +17414,8 @@
         <v>146</v>
       </c>
       <c r="V71" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y71,AA71,AC71,AE71,AG71)),1),"")</f>
-        <v>0.9</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y71,AA71,AC71,AE71,AG71)),1),0.4),"")</f>
+        <v>0.4</v>
       </c>
       <c r="W71" s="7" t="n">
         <f aca="false">COUNT(X71,Z71,AB71,AD71,AF71)</f>
@@ -17508,8 +17508,8 @@
         <v>147</v>
       </c>
       <c r="V72" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y72,AA72,AC72,AE72,AG72)),1),"")</f>
-        <v>0.7</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y72,AA72,AC72,AE72,AG72)),1),0.2),"")</f>
+        <v>0.2</v>
       </c>
       <c r="W72" s="7" t="n">
         <f aca="false">COUNT(X72,Z72,AB72,AD72,AF72)</f>
@@ -17995,7 +17995,7 @@
         <v>153</v>
       </c>
       <c r="V6" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y6,AA6,AC6,AE6,AG6)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y6,AA6,AC6,AE6,AG6)),1),70.5),"")</f>
         <v>69.4</v>
       </c>
       <c r="W6" s="7" t="n">
@@ -18104,7 +18104,7 @@
         <v>154</v>
       </c>
       <c r="V7" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y7,AA7,AC7,AE7,AG7)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y7,AA7,AC7,AE7,AG7)),1),69.8),"")</f>
         <v>68.1</v>
       </c>
       <c r="W7" s="7" t="n">
@@ -18220,7 +18220,7 @@
         <v>155</v>
       </c>
       <c r="V8" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y8,AA8,AC8,AE8,AG8)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y8,AA8,AC8,AE8,AG8)),1),66.3),"")</f>
         <v>64.8</v>
       </c>
       <c r="W8" s="7" t="n">
@@ -18336,7 +18336,7 @@
         <v>156</v>
       </c>
       <c r="V9" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y9,AA9,AC9,AE9,AG9)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y9,AA9,AC9,AE9,AG9)),1),65.9),"")</f>
         <v>64.8</v>
       </c>
       <c r="W9" s="7" t="n">
@@ -18452,7 +18452,7 @@
         <v>157</v>
       </c>
       <c r="V10" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y10,AA10,AC10,AE10,AG10)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y10,AA10,AC10,AE10,AG10)),1),55.6),"")</f>
         <v>54.5</v>
       </c>
       <c r="W10" s="7" t="n">
@@ -18568,7 +18568,7 @@
         <v>158</v>
       </c>
       <c r="V11" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y11,AA11,AC11,AE11,AG11)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y11,AA11,AC11,AE11,AG11)),1),52.2),"")</f>
         <v>51.1</v>
       </c>
       <c r="W11" s="7" t="n">
@@ -18684,7 +18684,7 @@
         <v>159</v>
       </c>
       <c r="V12" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y12,AA12,AC12,AE12,AG12)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y12,AA12,AC12,AE12,AG12)),1),47.4),"")</f>
         <v>46.7</v>
       </c>
       <c r="W12" s="7" t="n">
@@ -18800,7 +18800,7 @@
         <v>160</v>
       </c>
       <c r="V13" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y13,AA13,AC13,AE13,AG13)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y13,AA13,AC13,AE13,AG13)),1),47.3),"")</f>
         <v>46</v>
       </c>
       <c r="W13" s="7" t="n">
@@ -18916,7 +18916,7 @@
         <v>161</v>
       </c>
       <c r="V14" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y14,AA14,AC14,AE14,AG14)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y14,AA14,AC14,AE14,AG14)),1),45.7),"")</f>
         <v>45.2</v>
       </c>
       <c r="W14" s="7" t="n">
@@ -19032,7 +19032,7 @@
         <v>162</v>
       </c>
       <c r="V15" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y15,AA15,AC15,AE15,AG15)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y15,AA15,AC15,AE15,AG15)),1),44.5),"")</f>
         <v>44</v>
       </c>
       <c r="W15" s="7" t="n">
@@ -19148,7 +19148,7 @@
         <v>163</v>
       </c>
       <c r="V16" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y16,AA16,AC16,AE16,AG16)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y16,AA16,AC16,AE16,AG16)),1),43.4),"")</f>
         <v>42.4</v>
       </c>
       <c r="W16" s="7" t="n">
@@ -19264,7 +19264,7 @@
         <v>164</v>
       </c>
       <c r="V17" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y17,AA17,AC17,AE17,AG17)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y17,AA17,AC17,AE17,AG17)),1),41.9),"")</f>
         <v>40.4</v>
       </c>
       <c r="W17" s="7" t="n">
@@ -19380,7 +19380,7 @@
         <v>165</v>
       </c>
       <c r="V18" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y18,AA18,AC18,AE18,AG18)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y18,AA18,AC18,AE18,AG18)),1),39.9),"")</f>
         <v>39.3</v>
       </c>
       <c r="W18" s="7" t="n">
@@ -19489,7 +19489,7 @@
         <v>166</v>
       </c>
       <c r="V19" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y19,AA19,AC19,AE19,AG19)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y19,AA19,AC19,AE19,AG19)),1),38.2),"")</f>
         <v>37.4</v>
       </c>
       <c r="W19" s="7" t="n">
@@ -19591,7 +19591,7 @@
         <v>167</v>
       </c>
       <c r="V20" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y20,AA20,AC20,AE20,AG20)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y20,AA20,AC20,AE20,AG20)),1),37.6),"")</f>
         <v>36.4</v>
       </c>
       <c r="W20" s="7" t="n">
@@ -19693,7 +19693,7 @@
         <v>168</v>
       </c>
       <c r="V21" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y21,AA21,AC21,AE21,AG21)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y21,AA21,AC21,AE21,AG21)),1),34.1),"")</f>
         <v>33.2</v>
       </c>
       <c r="W21" s="7" t="n">
@@ -19795,7 +19795,7 @@
         <v>169</v>
       </c>
       <c r="V22" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y22,AA22,AC22,AE22,AG22)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y22,AA22,AC22,AE22,AG22)),1),33.4),"")</f>
         <v>33</v>
       </c>
       <c r="W22" s="7" t="n">
@@ -19897,7 +19897,7 @@
         <v>170</v>
       </c>
       <c r="V23" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y23,AA23,AC23,AE23,AG23)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y23,AA23,AC23,AE23,AG23)),1),33),"")</f>
         <v>31.9</v>
       </c>
       <c r="W23" s="7" t="n">
@@ -19999,7 +19999,7 @@
         <v>171</v>
       </c>
       <c r="V24" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y24,AA24,AC24,AE24,AG24)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y24,AA24,AC24,AE24,AG24)),1),32.2),"")</f>
         <v>31.3</v>
       </c>
       <c r="W24" s="7" t="n">
@@ -20101,7 +20101,7 @@
         <v>172</v>
       </c>
       <c r="V25" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y25,AA25,AC25,AE25,AG25)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y25,AA25,AC25,AE25,AG25)),1),30.4),"")</f>
         <v>29.5</v>
       </c>
       <c r="W25" s="7" t="n">
@@ -20203,7 +20203,7 @@
         <v>173</v>
       </c>
       <c r="V26" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y26,AA26,AC26,AE26,AG26)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y26,AA26,AC26,AE26,AG26)),1),30.3),"")</f>
         <v>29.4</v>
       </c>
       <c r="W26" s="7" t="n">
@@ -20305,7 +20305,7 @@
         <v>174</v>
       </c>
       <c r="V27" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y27,AA27,AC27,AE27,AG27)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y27,AA27,AC27,AE27,AG27)),1),29.1),"")</f>
         <v>28.2</v>
       </c>
       <c r="W27" s="7" t="n">
@@ -20407,7 +20407,7 @@
         <v>175</v>
       </c>
       <c r="V28" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y28,AA28,AC28,AE28,AG28)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y28,AA28,AC28,AE28,AG28)),1),26.5),"")</f>
         <v>26</v>
       </c>
       <c r="W28" s="7" t="n">
@@ -20509,7 +20509,7 @@
         <v>176</v>
       </c>
       <c r="V29" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y29,AA29,AC29,AE29,AG29)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y29,AA29,AC29,AE29,AG29)),1),25.8),"")</f>
         <v>24.6</v>
       </c>
       <c r="W29" s="7" t="n">
@@ -20611,7 +20611,7 @@
         <v>177</v>
       </c>
       <c r="V30" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y30,AA30,AC30,AE30,AG30)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y30,AA30,AC30,AE30,AG30)),1),25.5),"")</f>
         <v>25</v>
       </c>
       <c r="W30" s="7" t="n">
@@ -20713,7 +20713,7 @@
         <v>178</v>
       </c>
       <c r="V31" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y31,AA31,AC31,AE31,AG31)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y31,AA31,AC31,AE31,AG31)),1),25.4),"")</f>
         <v>24.2</v>
       </c>
       <c r="W31" s="7" t="n">
@@ -20815,7 +20815,7 @@
         <v>179</v>
       </c>
       <c r="V32" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y32,AA32,AC32,AE32,AG32)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y32,AA32,AC32,AE32,AG32)),1),25.4),"")</f>
         <v>24.3</v>
       </c>
       <c r="W32" s="7" t="n">
@@ -20917,7 +20917,7 @@
         <v>180</v>
       </c>
       <c r="V33" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y33,AA33,AC33,AE33,AG33)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y33,AA33,AC33,AE33,AG33)),1),25),"")</f>
         <v>24.2</v>
       </c>
       <c r="W33" s="7" t="n">
@@ -21019,7 +21019,7 @@
         <v>181</v>
       </c>
       <c r="V34" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y34,AA34,AC34,AE34,AG34)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y34,AA34,AC34,AE34,AG34)),1),22.8),"")</f>
         <v>22</v>
       </c>
       <c r="W34" s="7" t="n">
@@ -21121,7 +21121,7 @@
         <v>182</v>
       </c>
       <c r="V35" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y35,AA35,AC35,AE35,AG35)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y35,AA35,AC35,AE35,AG35)),1),20.9),"")</f>
         <v>19.9</v>
       </c>
       <c r="W35" s="7" t="n">
@@ -21223,7 +21223,7 @@
         <v>183</v>
       </c>
       <c r="V36" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y36,AA36,AC36,AE36,AG36)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y36,AA36,AC36,AE36,AG36)),1),18.6),"")</f>
         <v>17.7</v>
       </c>
       <c r="W36" s="7" t="n">
@@ -21325,7 +21325,7 @@
         <v>184</v>
       </c>
       <c r="V37" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y37,AA37,AC37,AE37,AG37)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y37,AA37,AC37,AE37,AG37)),1),18.6),"")</f>
         <v>17.8</v>
       </c>
       <c r="W37" s="7" t="n">
@@ -21427,7 +21427,7 @@
         <v>185</v>
       </c>
       <c r="V38" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y38,AA38,AC38,AE38,AG38)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y38,AA38,AC38,AE38,AG38)),1),18.4),"")</f>
         <v>17.7</v>
       </c>
       <c r="W38" s="7" t="n">
@@ -21529,7 +21529,7 @@
         <v>186</v>
       </c>
       <c r="V39" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y39,AA39,AC39,AE39,AG39)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y39,AA39,AC39,AE39,AG39)),1),18.3),"")</f>
         <v>17.1</v>
       </c>
       <c r="W39" s="7" t="n">
@@ -21631,7 +21631,7 @@
         <v>187</v>
       </c>
       <c r="V40" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y40,AA40,AC40,AE40,AG40)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y40,AA40,AC40,AE40,AG40)),1),16),"")</f>
         <v>15.1</v>
       </c>
       <c r="W40" s="7" t="n">
@@ -21733,7 +21733,7 @@
         <v>188</v>
       </c>
       <c r="V41" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y41,AA41,AC41,AE41,AG41)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y41,AA41,AC41,AE41,AG41)),1),14),"")</f>
         <v>13.2</v>
       </c>
       <c r="W41" s="7" t="n">
@@ -21835,7 +21835,7 @@
         <v>189</v>
       </c>
       <c r="V42" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y42,AA42,AC42,AE42,AG42)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y42,AA42,AC42,AE42,AG42)),1),13.5),"")</f>
         <v>13</v>
       </c>
       <c r="W42" s="7" t="n">
@@ -21935,7 +21935,7 @@
         <v>190</v>
       </c>
       <c r="V43" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y43,AA43,AC43,AE43,AG43)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y43,AA43,AC43,AE43,AG43)),1),12.7),"")</f>
         <v>12.5</v>
       </c>
       <c r="W43" s="7" t="n">
@@ -22035,7 +22035,7 @@
         <v>191</v>
       </c>
       <c r="V44" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y44,AA44,AC44,AE44,AG44)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y44,AA44,AC44,AE44,AG44)),1),12.2),"")</f>
         <v>12.1</v>
       </c>
       <c r="W44" s="7" t="n">
@@ -22137,7 +22137,7 @@
         <v>192</v>
       </c>
       <c r="V45" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y45,AA45,AC45,AE45,AG45)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y45,AA45,AC45,AE45,AG45)),1),11.6),"")</f>
         <v>11.3</v>
       </c>
       <c r="W45" s="7" t="n">
@@ -22239,8 +22239,8 @@
         <v>193</v>
       </c>
       <c r="V46" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y46,AA46,AC46,AE46,AG46)),1),"")</f>
-        <v>12.3</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y46,AA46,AC46,AE46,AG46)),1),11.6),"")</f>
+        <v>11.6</v>
       </c>
       <c r="W46" s="7" t="n">
         <f aca="false">COUNT(X46,Z46,AB46,AD46,AF46)</f>
@@ -22339,8 +22339,8 @@
         <v>194</v>
       </c>
       <c r="V47" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y47,AA47,AC47,AE47,AG47)),1),"")</f>
-        <v>12.5</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y47,AA47,AC47,AE47,AG47)),1),11.5),"")</f>
+        <v>11.5</v>
       </c>
       <c r="W47" s="7" t="n">
         <f aca="false">COUNT(X47,Z47,AB47,AD47,AF47)</f>
@@ -22439,7 +22439,7 @@
         <v>195</v>
       </c>
       <c r="V48" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y48,AA48,AC48,AE48,AG48)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y48,AA48,AC48,AE48,AG48)),1),10.9),"")</f>
         <v>10</v>
       </c>
       <c r="W48" s="7" t="n">
@@ -22541,8 +22541,8 @@
         <v>196</v>
       </c>
       <c r="V49" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y49,AA49,AC49,AE49,AG49)),1),"")</f>
-        <v>11.5</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y49,AA49,AC49,AE49,AG49)),1),10.8),"")</f>
+        <v>10.8</v>
       </c>
       <c r="W49" s="7" t="n">
         <f aca="false">COUNT(X49,Z49,AB49,AD49,AF49)</f>
@@ -22643,7 +22643,7 @@
         <v>197</v>
       </c>
       <c r="V50" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y50,AA50,AC50,AE50,AG50)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y50,AA50,AC50,AE50,AG50)),1),10.5),"")</f>
         <v>10.2</v>
       </c>
       <c r="W50" s="7" t="n">
@@ -22745,7 +22745,7 @@
         <v>198</v>
       </c>
       <c r="V51" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y51,AA51,AC51,AE51,AG51)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y51,AA51,AC51,AE51,AG51)),1),10.4),"")</f>
         <v>8.1</v>
       </c>
       <c r="W51" s="7" t="n">
@@ -22847,7 +22847,7 @@
         <v>199</v>
       </c>
       <c r="V52" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y52,AA52,AC52,AE52,AG52)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y52,AA52,AC52,AE52,AG52)),1),10.2),"")</f>
         <v>9.9</v>
       </c>
       <c r="W52" s="7" t="n">
@@ -22949,7 +22949,7 @@
         <v>200</v>
       </c>
       <c r="V53" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y53,AA53,AC53,AE53,AG53)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y53,AA53,AC53,AE53,AG53)),1),9.5),"")</f>
         <v>8.8</v>
       </c>
       <c r="W53" s="7" t="n">
@@ -23051,8 +23051,8 @@
         <v>201</v>
       </c>
       <c r="V54" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y54,AA54,AC54,AE54,AG54)),1),"")</f>
-        <v>8.9</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y54,AA54,AC54,AE54,AG54)),1),8.2),"")</f>
+        <v>8.2</v>
       </c>
       <c r="W54" s="7" t="n">
         <f aca="false">COUNT(X54,Z54,AB54,AD54,AF54)</f>
@@ -23153,7 +23153,7 @@
         <v>202</v>
       </c>
       <c r="V55" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y55,AA55,AC55,AE55,AG55)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y55,AA55,AC55,AE55,AG55)),1),7.9),"")</f>
         <v>7.3</v>
       </c>
       <c r="W55" s="7" t="n">
@@ -23255,7 +23255,7 @@
         <v>203</v>
       </c>
       <c r="V56" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y56,AA56,AC56,AE56,AG56)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y56,AA56,AC56,AE56,AG56)),1),7.3),"")</f>
         <v>6.3</v>
       </c>
       <c r="W56" s="7" t="n">
@@ -23353,7 +23353,7 @@
         <v>204</v>
       </c>
       <c r="V57" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y57,AA57,AC57,AE57,AG57)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y57,AA57,AC57,AE57,AG57)),1),7.2),"")</f>
         <v>6.6</v>
       </c>
       <c r="W57" s="7" t="n">
@@ -23447,8 +23447,8 @@
         <v>205</v>
       </c>
       <c r="V58" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y58,AA58,AC58,AE58,AG58)),1),"")</f>
-        <v>7.4</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y58,AA58,AC58,AE58,AG58)),1),6.9),"")</f>
+        <v>6.9</v>
       </c>
       <c r="W58" s="7" t="n">
         <f aca="false">COUNT(X58,Z58,AB58,AD58,AF58)</f>
@@ -23545,8 +23545,8 @@
         <v>206</v>
       </c>
       <c r="V59" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y59,AA59,AC59,AE59,AG59)),1),"")</f>
-        <v>7.3</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y59,AA59,AC59,AE59,AG59)),1),6.6),"")</f>
+        <v>6.6</v>
       </c>
       <c r="W59" s="7" t="n">
         <f aca="false">COUNT(X59,Z59,AB59,AD59,AF59)</f>
@@ -23645,8 +23645,8 @@
         <v>207</v>
       </c>
       <c r="V60" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y60,AA60,AC60,AE60,AG60)),1),"")</f>
-        <v>7</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y60,AA60,AC60,AE60,AG60)),1),6.2),"")</f>
+        <v>6.2</v>
       </c>
       <c r="W60" s="7" t="n">
         <f aca="false">COUNT(X60,Z60,AB60,AD60,AF60)</f>
@@ -23745,8 +23745,8 @@
         <v>208</v>
       </c>
       <c r="V61" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y61,AA61,AC61,AE61,AG61)),1),"")</f>
-        <v>6.8</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y61,AA61,AC61,AE61,AG61)),1),5.9),"")</f>
+        <v>5.9</v>
       </c>
       <c r="W61" s="7" t="n">
         <f aca="false">COUNT(X61,Z61,AB61,AD61,AF61)</f>
@@ -23845,8 +23845,8 @@
         <v>209</v>
       </c>
       <c r="V62" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y62,AA62,AC62,AE62,AG62)),1),"")</f>
-        <v>6.4</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y62,AA62,AC62,AE62,AG62)),1),5.7),"")</f>
+        <v>5.7</v>
       </c>
       <c r="W62" s="7" t="n">
         <f aca="false">COUNT(X62,Z62,AB62,AD62,AF62)</f>
@@ -23941,7 +23941,7 @@
         <v>210</v>
       </c>
       <c r="V63" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y63,AA63,AC63,AE63,AG63)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y63,AA63,AC63,AE63,AG63)),1),5.2),"")</f>
         <v>3.8</v>
       </c>
       <c r="W63" s="7" t="n">
@@ -24035,7 +24035,7 @@
         <v>211</v>
       </c>
       <c r="V64" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y64,AA64,AC64,AE64,AG64)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y64,AA64,AC64,AE64,AG64)),1),4.9),"")</f>
         <v>3.9</v>
       </c>
       <c r="W64" s="7" t="n">
@@ -24131,8 +24131,8 @@
         <v>212</v>
       </c>
       <c r="V65" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y65,AA65,AC65,AE65,AG65)),1),"")</f>
-        <v>5.6</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y65,AA65,AC65,AE65,AG65)),1),4.9),"")</f>
+        <v>4.9</v>
       </c>
       <c r="W65" s="7" t="n">
         <f aca="false">COUNT(X65,Z65,AB65,AD65,AF65)</f>
@@ -24227,7 +24227,7 @@
         <v>213</v>
       </c>
       <c r="V66" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y66,AA66,AC66,AE66,AG66)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y66,AA66,AC66,AE66,AG66)),1),4.1),"")</f>
         <v>4</v>
       </c>
       <c r="W66" s="7" t="n">
@@ -24321,8 +24321,8 @@
         <v>214</v>
       </c>
       <c r="V67" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y67,AA67,AC67,AE67,AG67)),1),"")</f>
-        <v>4.3</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y67,AA67,AC67,AE67,AG67)),1),3.9),"")</f>
+        <v>3.9</v>
       </c>
       <c r="W67" s="7" t="n">
         <f aca="false">COUNT(X67,Z67,AB67,AD67,AF67)</f>
@@ -24417,8 +24417,8 @@
         <v>215</v>
       </c>
       <c r="V68" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y68,AA68,AC68,AE68,AG68)),1),"")</f>
-        <v>4.3</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y68,AA68,AC68,AE68,AG68)),1),3.9),"")</f>
+        <v>3.9</v>
       </c>
       <c r="W68" s="7" t="n">
         <f aca="false">COUNT(X68,Z68,AB68,AD68,AF68)</f>
@@ -24511,7 +24511,7 @@
         <v>216</v>
       </c>
       <c r="V69" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y69,AA69,AC69,AE69,AG69)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y69,AA69,AC69,AE69,AG69)),1),3.7),"")</f>
         <v>3.5</v>
       </c>
       <c r="W69" s="7" t="n">
@@ -24605,7 +24605,7 @@
         <v>217</v>
       </c>
       <c r="V70" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y70,AA70,AC70,AE70,AG70)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y70,AA70,AC70,AE70,AG70)),1),3.6),"")</f>
         <v>3.5</v>
       </c>
       <c r="W70" s="7" t="n">
@@ -24701,8 +24701,8 @@
         <v>218</v>
       </c>
       <c r="V71" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y71,AA71,AC71,AE71,AG71)),1),"")</f>
-        <v>3.9</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y71,AA71,AC71,AE71,AG71)),1),3.2),"")</f>
+        <v>3.2</v>
       </c>
       <c r="W71" s="7" t="n">
         <f aca="false">COUNT(X71,Z71,AB71,AD71,AF71)</f>
@@ -24799,8 +24799,8 @@
         <v>219</v>
       </c>
       <c r="V72" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y72,AA72,AC72,AE72,AG72)),1),"")</f>
-        <v>3.7</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y72,AA72,AC72,AE72,AG72)),1),3),"")</f>
+        <v>3</v>
       </c>
       <c r="W72" s="7" t="n">
         <f aca="false">COUNT(X72,Z72,AB72,AD72,AF72)</f>
@@ -24895,7 +24895,7 @@
         <v>220</v>
       </c>
       <c r="V73" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y73,AA73,AC73,AE73,AG73)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y73,AA73,AC73,AE73,AG73)),1),2.8),"")</f>
         <v>2.6</v>
       </c>
       <c r="W73" s="7" t="n">
@@ -24991,8 +24991,8 @@
         <v>221</v>
       </c>
       <c r="V74" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y74,AA74,AC74,AE74,AG74)),1),"")</f>
-        <v>3.5</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y74,AA74,AC74,AE74,AG74)),1),2.8),"")</f>
+        <v>2.8</v>
       </c>
       <c r="W74" s="7" t="n">
         <f aca="false">COUNT(X74,Z74,AB74,AD74,AF74)</f>
@@ -25089,8 +25089,8 @@
         <v>222</v>
       </c>
       <c r="V75" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y75,AA75,AC75,AE75,AG75)),1),"")</f>
-        <v>3</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y75,AA75,AC75,AE75,AG75)),1),2.4),"")</f>
+        <v>2.4</v>
       </c>
       <c r="W75" s="7" t="n">
         <f aca="false">COUNT(X75,Z75,AB75,AD75,AF75)</f>
@@ -25185,7 +25185,7 @@
         <v>224</v>
       </c>
       <c r="V76" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y76,AA76,AC76,AE76,AG76)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y76,AA76,AC76,AE76,AG76)),1),1.9),"")</f>
         <v>0.1</v>
       </c>
       <c r="W76" s="7" t="n">
@@ -25279,8 +25279,8 @@
         <v>225</v>
       </c>
       <c r="V77" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y77,AA77,AC77,AE77,AG77)),1),"")</f>
-        <v>2.2</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y77,AA77,AC77,AE77,AG77)),1),1.6),"")</f>
+        <v>1.6</v>
       </c>
       <c r="W77" s="7" t="n">
         <f aca="false">COUNT(X77,Z77,AB77,AD77,AF77)</f>
@@ -25375,8 +25375,8 @@
         <v>227</v>
       </c>
       <c r="V78" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y78,AA78,AC78,AE78,AG78)),1),"")</f>
-        <v>1.8</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y78,AA78,AC78,AE78,AG78)),1),1.4),"")</f>
+        <v>1.4</v>
       </c>
       <c r="W78" s="7" t="n">
         <f aca="false">COUNT(X78,Z78,AB78,AD78,AF78)</f>
@@ -25471,8 +25471,8 @@
         <v>228</v>
       </c>
       <c r="V79" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y79,AA79,AC79,AE79,AG79)),1),"")</f>
-        <v>1.9</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y79,AA79,AC79,AE79,AG79)),1),1.2),"")</f>
+        <v>1.2</v>
       </c>
       <c r="W79" s="7" t="n">
         <f aca="false">COUNT(X79,Z79,AB79,AD79,AF79)</f>
@@ -25567,8 +25567,8 @@
         <v>230</v>
       </c>
       <c r="V80" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y80,AA80,AC80,AE80,AG80)),1),"")</f>
-        <v>1.3</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y80,AA80,AC80,AE80,AG80)),1),1.1),"")</f>
+        <v>1.1</v>
       </c>
       <c r="W80" s="7" t="n">
         <f aca="false">COUNT(X80,Z80,AB80,AD80,AF80)</f>
@@ -25661,8 +25661,8 @@
         <v>231</v>
       </c>
       <c r="V81" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y81,AA81,AC81,AE81,AG81)),1),"")</f>
-        <v>1.8</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y81,AA81,AC81,AE81,AG81)),1),1.1),"")</f>
+        <v>1.1</v>
       </c>
       <c r="W81" s="7" t="n">
         <f aca="false">COUNT(X81,Z81,AB81,AD81,AF81)</f>
@@ -25759,8 +25759,8 @@
         <v>232</v>
       </c>
       <c r="V82" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y82,AA82,AC82,AE82,AG82)),1),"")</f>
-        <v>1.2</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y82,AA82,AC82,AE82,AG82)),1),1.1),"")</f>
+        <v>1.1</v>
       </c>
       <c r="W82" s="7" t="n">
         <f aca="false">COUNT(X82,Z82,AB82,AD82,AF82)</f>
@@ -25853,8 +25853,8 @@
         <v>233</v>
       </c>
       <c r="V83" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y83,AA83,AC83,AE83,AG83)),1),"")</f>
-        <v>1.5</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y83,AA83,AC83,AE83,AG83)),1),0.8),"")</f>
+        <v>0.8</v>
       </c>
       <c r="W83" s="7" t="n">
         <f aca="false">COUNT(X83,Z83,AB83,AD83,AF83)</f>
@@ -25951,8 +25951,8 @@
         <v>234</v>
       </c>
       <c r="V84" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y84,AA84,AC84,AE84,AG84)),1),"")</f>
-        <v>1.1</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y84,AA84,AC84,AE84,AG84)),1),0.5),"")</f>
+        <v>0.5</v>
       </c>
       <c r="W84" s="7" t="n">
         <f aca="false">COUNT(X84,Z84,AB84,AD84,AF84)</f>
@@ -26047,8 +26047,8 @@
         <v>235</v>
       </c>
       <c r="V85" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y85,AA85,AC85,AE85,AG85)),1),"")</f>
-        <v>0.6</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y85,AA85,AC85,AE85,AG85)),1),0.4),"")</f>
+        <v>0.4</v>
       </c>
       <c r="W85" s="7" t="n">
         <f aca="false">COUNT(X85,Z85,AB85,AD85,AF85)</f>
@@ -26143,8 +26143,8 @@
         <v>236</v>
       </c>
       <c r="V86" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y86,AA86,AC86,AE86,AG86)),1),"")</f>
-        <v>0.3</v>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y86,AA86,AC86,AE86,AG86)),1),0),"")</f>
+        <v>0</v>
       </c>
       <c r="W86" s="7" t="n">
         <f aca="false">COUNT(X86,Z86,AB86,AD86,AF86)</f>
@@ -26241,7 +26241,7 @@
         <v>237</v>
       </c>
       <c r="V87" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y87,AA87,AC87,AE87,AG87)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y87,AA87,AC87,AE87,AG87)),1),0),"")</f>
         <v>0</v>
       </c>
       <c r="W87" s="7" t="n">
@@ -26636,7 +26636,7 @@
         <v>241</v>
       </c>
       <c r="V6" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y6,AA6,AC6,AE6,AG6)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y6,AA6,AC6,AE6,AG6)),1),42.5),"")</f>
         <v>40.8</v>
       </c>
       <c r="W6" s="7" t="n">
@@ -26745,7 +26745,7 @@
         <v>242</v>
       </c>
       <c r="V7" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y7,AA7,AC7,AE7,AG7)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y7,AA7,AC7,AE7,AG7)),1),37.9),"")</f>
         <v>35.3</v>
       </c>
       <c r="W7" s="7" t="n">
@@ -26861,7 +26861,7 @@
         <v>243</v>
       </c>
       <c r="V8" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y8,AA8,AC8,AE8,AG8)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y8,AA8,AC8,AE8,AG8)),1),31.3),"")</f>
         <v>29.7</v>
       </c>
       <c r="W8" s="7" t="n">
@@ -26977,7 +26977,7 @@
         <v>244</v>
       </c>
       <c r="V9" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y9,AA9,AC9,AE9,AG9)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y9,AA9,AC9,AE9,AG9)),1),22.4),"")</f>
         <v>21.4</v>
       </c>
       <c r="W9" s="7" t="n">
@@ -27093,7 +27093,7 @@
         <v>245</v>
       </c>
       <c r="V10" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y10,AA10,AC10,AE10,AG10)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y10,AA10,AC10,AE10,AG10)),1),19.1),"")</f>
         <v>18</v>
       </c>
       <c r="W10" s="7" t="n">
@@ -27209,7 +27209,7 @@
         <v>246</v>
       </c>
       <c r="V11" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y11,AA11,AC11,AE11,AG11)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y11,AA11,AC11,AE11,AG11)),1),16),"")</f>
         <v>14.9</v>
       </c>
       <c r="W11" s="7" t="n">
@@ -27325,7 +27325,7 @@
         <v>247</v>
       </c>
       <c r="V12" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y12,AA12,AC12,AE12,AG12)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y12,AA12,AC12,AE12,AG12)),1),13.7),"")</f>
         <v>12.4</v>
       </c>
       <c r="W12" s="7" t="n">
@@ -27441,7 +27441,7 @@
         <v>248</v>
       </c>
       <c r="V13" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y13,AA13,AC13,AE13,AG13)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y13,AA13,AC13,AE13,AG13)),1),13.5),"")</f>
         <v>12.5</v>
       </c>
       <c r="W13" s="7" t="n">
@@ -27557,7 +27557,7 @@
         <v>249</v>
       </c>
       <c r="V14" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y14,AA14,AC14,AE14,AG14)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y14,AA14,AC14,AE14,AG14)),1),13.5),"")</f>
         <v>11.9</v>
       </c>
       <c r="W14" s="7" t="n">
@@ -27673,7 +27673,7 @@
         <v>250</v>
       </c>
       <c r="V15" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y15,AA15,AC15,AE15,AG15)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y15,AA15,AC15,AE15,AG15)),1),9),"")</f>
         <v>7.9</v>
       </c>
       <c r="W15" s="7" t="n">
@@ -27789,7 +27789,7 @@
         <v>251</v>
       </c>
       <c r="V16" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y16,AA16,AC16,AE16,AG16)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y16,AA16,AC16,AE16,AG16)),1),8.4),"")</f>
         <v>8.1</v>
       </c>
       <c r="W16" s="7" t="n">
@@ -27903,7 +27903,7 @@
         <v>252</v>
       </c>
       <c r="V17" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y17,AA17,AC17,AE17,AG17)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y17,AA17,AC17,AE17,AG17)),1),8.2),"")</f>
         <v>6.4</v>
       </c>
       <c r="W17" s="7" t="n">
@@ -28015,7 +28015,7 @@
         <v>253</v>
       </c>
       <c r="V18" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y18,AA18,AC18,AE18,AG18)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y18,AA18,AC18,AE18,AG18)),1),8),"")</f>
         <v>5.4</v>
       </c>
       <c r="W18" s="7" t="n">
@@ -28120,7 +28120,7 @@
         <v>254</v>
       </c>
       <c r="V19" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y19,AA19,AC19,AE19,AG19)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y19,AA19,AC19,AE19,AG19)),1),6.1),"")</f>
         <v>5.8</v>
       </c>
       <c r="W19" s="7" t="n">
@@ -28218,7 +28218,7 @@
         <v>255</v>
       </c>
       <c r="V20" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y20,AA20,AC20,AE20,AG20)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y20,AA20,AC20,AE20,AG20)),1),5.5),"")</f>
         <v>4.5</v>
       </c>
       <c r="W20" s="7" t="n">
@@ -28314,7 +28314,7 @@
         <v>256</v>
       </c>
       <c r="V21" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y21,AA21,AC21,AE21,AG21)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y21,AA21,AC21,AE21,AG21)),1),4.9),"")</f>
         <v>3.7</v>
       </c>
       <c r="W21" s="7" t="n">
@@ -28410,7 +28410,7 @@
         <v>257</v>
       </c>
       <c r="V22" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y22,AA22,AC22,AE22,AG22)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y22,AA22,AC22,AE22,AG22)),1),4.7),"")</f>
         <v>2.9</v>
       </c>
       <c r="W22" s="7" t="n">
@@ -28506,7 +28506,7 @@
         <v>258</v>
       </c>
       <c r="V23" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y23,AA23,AC23,AE23,AG23)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y23,AA23,AC23,AE23,AG23)),1),4.7),"")</f>
         <v>3.5</v>
       </c>
       <c r="W23" s="7" t="n">
@@ -28600,7 +28600,7 @@
         <v>259</v>
       </c>
       <c r="V24" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y24,AA24,AC24,AE24,AG24)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y24,AA24,AC24,AE24,AG24)),1),4.1),"")</f>
         <v>0.2</v>
       </c>
       <c r="W24" s="7" t="n">
@@ -28696,7 +28696,7 @@
         <v>260</v>
       </c>
       <c r="V25" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y25,AA25,AC25,AE25,AG25)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y25,AA25,AC25,AE25,AG25)),1),3.8),"")</f>
         <v>3.4</v>
       </c>
       <c r="W25" s="7" t="n">
@@ -28792,7 +28792,7 @@
         <v>262</v>
       </c>
       <c r="V26" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y26,AA26,AC26,AE26,AG26)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y26,AA26,AC26,AE26,AG26)),1),3.6),"")</f>
         <v>2.5</v>
       </c>
       <c r="W26" s="7" t="n">
@@ -28886,7 +28886,7 @@
         <v>263</v>
       </c>
       <c r="V27" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y27,AA27,AC27,AE27,AG27)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y27,AA27,AC27,AE27,AG27)),1),3.5),"")</f>
         <v>1.4</v>
       </c>
       <c r="W27" s="7" t="n">
@@ -28980,7 +28980,7 @@
         <v>264</v>
       </c>
       <c r="V28" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y28,AA28,AC28,AE28,AG28)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y28,AA28,AC28,AE28,AG28)),1),3.4),"")</f>
         <v>1.4</v>
       </c>
       <c r="W28" s="7" t="n">
@@ -29074,7 +29074,7 @@
         <v>265</v>
       </c>
       <c r="V29" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y29,AA29,AC29,AE29,AG29)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y29,AA29,AC29,AE29,AG29)),1),3.3),"")</f>
         <v>2.6</v>
       </c>
       <c r="W29" s="7" t="n">
@@ -29168,7 +29168,7 @@
         <v>266</v>
       </c>
       <c r="V30" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y30,AA30,AC30,AE30,AG30)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y30,AA30,AC30,AE30,AG30)),1),2.1),"")</f>
         <v>1.7</v>
       </c>
       <c r="W30" s="7" t="n">
@@ -29266,7 +29266,7 @@
         <v>268</v>
       </c>
       <c r="V31" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y31,AA31,AC31,AE31,AG31)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y31,AA31,AC31,AE31,AG31)),1),2.1),"")</f>
         <v>1.3</v>
       </c>
       <c r="W31" s="7" t="n">
@@ -29364,7 +29364,7 @@
         <v>269</v>
       </c>
       <c r="V32" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y32,AA32,AC32,AE32,AG32)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y32,AA32,AC32,AE32,AG32)),1),1.9),"")</f>
         <v>1.2</v>
       </c>
       <c r="W32" s="7" t="n">
@@ -29458,7 +29458,7 @@
         <v>270</v>
       </c>
       <c r="V33" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y33,AA33,AC33,AE33,AG33)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y33,AA33,AC33,AE33,AG33)),1),1.9),"")</f>
         <v>1.1</v>
       </c>
       <c r="W33" s="7" t="n">
@@ -29552,7 +29552,7 @@
         <v>272</v>
       </c>
       <c r="V34" s="6" t="n">
-        <f aca="false">IFERROR(ROUND(MAX(0,AVERAGE(Y34,AA34,AC34,AE34,AG34)),1),"")</f>
+        <f aca="false">IFERROR(MIN(ROUND(MAX(0,AVERAGE(Y34,AA34,AC34,AE34,AG34)),1),1.6),"")</f>
         <v>0.8</v>
       </c>
       <c r="W34" s="7" t="n">

</xml_diff>